<commit_message>
fix: corrige seletor de datas, sincronização de períodos e adiciona validação de dados em C5
- Pré-popula o seletor de meses no HTML com todas as opções
- Alinha os dados mensais de receitas e despesas registradas para cada mês selecionado
- Atualiza todos os componentes, notas e períodos ao alterar o seletor ou carregar planilha
- Adiciona lista suspensa (Validação de Dados) na célula C5 do Dashboard na planilha Excel
</commit_message>
<xml_diff>
--- a/CONTROLE-FINANCEIRO JM.xlsx
+++ b/CONTROLE-FINANCEIRO JM.xlsx
@@ -6362,6 +6362,11 @@
     <mergeCell ref="E52:M53"/>
     <mergeCell ref="E55:M57"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" sqref="C5">
+      <formula1>"Janeiro/2026,Fevereiro/2026,Março/2026,Abril/2026,Maio/2026,Junho/2026,Julho/2026,Agosto/2026,Setembro/2026,Outubro/2026,Novembro/2026,Dezembro/2026"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="H30" location="PATRIMÔNIO!A1" display="→ PATRIMÔNIO" ns2:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="H29" location="'CONTROLE LANCAMENTOS'!A1" display="'CONTROLE LANCAMENTOS'!A1" ns2:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>